<commit_message>
Translation review sheet: 69 strings (adds the two confidence labels and the app's copy/share wording)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/review/translation-review-2026-10.xlsx
+++ b/docs/review/translation-review-2026-10.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Strings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Strings'!$A$1:$N$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Strings'!$A$1:$N$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Strings new or changed between origin/main and origin/scan-error-codes that farmers see (web and app).</t>
+          <t>Strings new or changed between 5e2b726b9 and HEAD that farmers see (web and app).</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -601,7 +601,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Nutrients, Recommendations</t>
+          <t>No single finding</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -611,36 +611,36 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Nutrients, Recommendations</t>
+          <t>No single finding</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Abubuwan Gina Jiki da Shawarwari</t>
+          <t>Babu sakamako guda ɗaya</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Àwọn ohun oúnjẹ, Àwọn ìmọ̀ràn</t>
+          <t>Kò sí àbájáde kan pàtó</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Nri, Ndụmọdụ</t>
+          <t>Enweghị otu nchọpụta</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Nutriments, Recommandations</t>
+          <t>Pas de résultat unique</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>المغذيات، التوصيات</t>
+          <t>لا توجد نتيجة واحدة</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr"/>
@@ -653,7 +653,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Not certain</t>
+          <t>AI Analysis Unavailable</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -663,36 +663,36 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Not certain</t>
+          <t>AI Analysis Unavailable</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Ba a tabbata ba</t>
+          <t>Binciken AI bai samu ba</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Kò dájú</t>
+          <t>Àyẹ̀wò AI kò sí</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>O doghị anya</t>
+          <t>Nyocha AI adịghị</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Pas certain</t>
+          <t>Analyse IA indisponible</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>غير مؤكد</t>
+          <t>تحليل الذكاء الاصطناعي غير متاح</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr"/>
@@ -705,7 +705,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Likely</t>
+          <t>Nutrients, Recommendations</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -715,36 +715,36 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Likely</t>
+          <t>Nutrients, Recommendations</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Wataƙila</t>
+          <t>Abubuwan Gina Jiki da Shawarwari</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>Àwọn ohun oúnjẹ, Àwọn ìmọ̀ràn</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>Nri, Ndụmọdụ</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Probable</t>
+          <t>Nutriments, Recommandations</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>المغذيات، التوصيات</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr"/>
@@ -757,7 +757,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>The AI thinks this is likely, but is not fully sure. Please confirm with a vet or extension officer before treating.</t>
+          <t>Not certain</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -767,36 +767,36 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>The AI thinks this is likely, but is not fully sure. Please confirm with a vet or extension officer before treating.</t>
+          <t>Not certain</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>AI na ganin hakan ne mai yiwuwa, amma bai tabbata sosai ba. Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
+          <t>Ba a tabbata ba</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>Kò dájú</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>O doghị anya</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>L'IA pense que c'est probable, mais n'en est pas tout à fait sûre. Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
+          <t>Pas certain</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>غير مؤكد</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr"/>
@@ -809,7 +809,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>The AI is not sure enough to give one diagnosis. These are the possible conditions:</t>
+          <t>Likely</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -819,36 +819,36 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>The AI is not sure enough to give one diagnosis. These are the possible conditions:</t>
+          <t>Likely</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>AI ba ta da isasshen tabbaci don ba da cuta ɗaya. Ga cututtukan da za su iya kasancewa:</t>
+          <t>Wataƙila</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>AI kò ní ìdánilójú tó láti fún ọ ní àrùn kan ṣoṣo. Àwọn àrùn tó ṣeé ṣe nìwọ̀nyí:</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>AI enweghị ezigbo ntụkwasị obi iji kwuo otu ọrịa. Ndị a bụ ọrịa ndị nwere ike ịbụ:</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>L'IA n'est pas assez sûre pour donner un seul diagnostic. Voici les problèmes possibles :</t>
+          <t>Probable</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>الذكاء الاصطناعي غير متأكد بما يكفي لإعطاء تشخيص واحد. هذه هي الحالات المحتملة:</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr"/>
@@ -861,7 +861,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Possible conditions</t>
+          <t>The AI thinks this is likely, but is not fully sure. Please confirm with a vet or extension officer before treating.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -871,36 +871,36 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Possible conditions</t>
+          <t>The AI thinks this is likely, but is not fully sure. Please confirm with a vet or extension officer before treating.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Cututtukan da za su iya kasancewa</t>
+          <t>AI na ganin hakan ne mai yiwuwa, amma bai tabbata sosai ba. Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Àwọn àrùn tó ṣeé ṣe</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Ọrịa ndị nwere ike ịbụ</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Problèmes possibles</t>
+          <t>L'IA pense que c'est probable, mais n'en est pas tout à fait sûre. Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>الحالات المحتملة</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr"/>
@@ -913,7 +913,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Please confirm with a vet or extension officer before treating.</t>
+          <t>The AI is not sure enough to give one diagnosis. These are the possible conditions:</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -923,36 +923,36 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Please confirm with a vet or extension officer before treating.</t>
+          <t>The AI is not sure enough to give one diagnosis. These are the possible conditions:</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
+          <t>AI ba ta da isasshen tabbaci don ba da cuta ɗaya. Ga cututtukan da za su iya kasancewa:</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Jọ̀wọ́ fìdí rẹ̀ múlẹ̀ pẹ̀lú dókítà ẹranko tàbí òṣìṣẹ́ àgbẹ̀ kí o tó tọ́jú.</t>
+          <t>AI kò ní ìdánilójú tó láti fún ọ ní àrùn kan ṣoṣo. Àwọn àrùn tó ṣeé ṣe nìwọ̀nyí:</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Biko kwado ya na dọkịta anụmanụ ma ọ bụ onye ndụmọdụ ugbo tupu ị gwọọ.</t>
+          <t>AI enweghị ezigbo ntụkwasị obi iji kwuo otu ọrịa. Ndị a bụ ọrịa ndị nwere ike ịbụ:</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
+          <t>L'IA n'est pas assez sûre pour donner un seul diagnostic. Voici les problèmes possibles :</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>يرجى التأكد من طبيب بيطري أو مرشد زراعي قبل العلاج.</t>
+          <t>الذكاء الاصطناعي غير متأكد بما يكفي لإعطاء تشخيص واحد. هذه هي الحالات المحتملة:</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr"/>
@@ -965,7 +965,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>AI guidance can be wrong; confirm with an expert.</t>
+          <t>Possible conditions</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -975,36 +975,36 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>AI guidance can be wrong; confirm with an expert.</t>
+          <t>Possible conditions</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Shawarar AI na iya yin kuskure; ka tabbatar da ƙwararre.</t>
+          <t>Cututtukan da za su iya kasancewa</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Ìmọ̀ràn AI lè ṣàṣìṣe; fìdí rẹ̀ múlẹ̀ pẹ̀lú amòye.</t>
+          <t>Àwọn àrùn tó ṣeé ṣe</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Ndụmọdụ AI nwere ike ihie ụzọ; kwado ya na ọkachamara.</t>
+          <t>Ọrịa ndị nwere ike ịbụ</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Les conseils de l'IA peuvent être erronés ; confirmez auprès d'un expert.</t>
+          <t>Problèmes possibles</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>قد تكون إرشادات الذكاء الاصطناعي خاطئة؛ تأكد مع خبير.</t>
+          <t>الحالات المحتملة</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr"/>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>JPG, PNG, WebP or HEIC, up to 10 MB</t>
+          <t>Please confirm with a vet or extension officer before treating.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1027,36 +1027,36 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>JPG, PNG, WebP or HEIC, up to 10 MB</t>
+          <t>Please confirm with a vet or extension officer before treating.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>JPG, PNG, WebP ko HEIC, har zuwa 10 MB</t>
+          <t>Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>JPG, PNG, WebP tàbí HEIC, títí dé 10 MB</t>
+          <t>Jọ̀wọ́ fìdí rẹ̀ múlẹ̀ pẹ̀lú dókítà ẹranko tàbí òṣìṣẹ́ àgbẹ̀ kí o tó tọ́jú.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>JPG, PNG, WebP ma ọ bụ HEIC, ruo 10 MB</t>
+          <t>Biko kwado ya na dọkịta anụmanụ ma ọ bụ onye ndụmọdụ ugbo tupu ị gwọọ.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>JPG, PNG, WebP ou HEIC, jusqu'à 10 Mo</t>
+          <t>Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>JPG أو PNG أو WebP أو HEIC، حتى 10 ميغابايت</t>
+          <t>يرجى التأكد من طبيب بيطري أو مرشد زراعي قبل العلاج.</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr"/>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>This file type is not supported. Choose a JPG, PNG, WebP or HEIC photo.</t>
+          <t>AI guidance can be wrong; confirm with an expert.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1079,36 +1079,36 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>This file type is not supported. Choose a JPG, PNG, WebP or HEIC photo.</t>
+          <t>AI guidance can be wrong; confirm with an expert.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Ba a karɓar irin wannan fayil ba. Zaɓi hoton JPG, PNG, WebP ko HEIC.</t>
+          <t>Shawarar AI na iya yin kuskure; ka tabbatar da ƙwararre.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>A kò gba irú fáìlì yìí. Yan fọ́tò JPG, PNG, WebP tàbí HEIC.</t>
+          <t>Ìmọ̀ràn AI lè ṣàṣìṣe; fìdí rẹ̀ múlẹ̀ pẹ̀lú amòye.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Anaghị anabata ụdị faịlụ a. Họrọ foto JPG, PNG, WebP ma ọ bụ HEIC.</t>
+          <t>Ndụmọdụ AI nwere ike ihie ụzọ; kwado ya na ọkachamara.</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Ce type de fichier n'est pas pris en charge. Choisissez une photo JPG, PNG, WebP ou HEIC.</t>
+          <t>Les conseils de l'IA peuvent être erronés ; confirmez auprès d'un expert.</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>نوع الملف هذا غير مدعوم. اختر صورة JPG أو PNG أو WebP أو HEIC.</t>
+          <t>قد تكون إرشادات الذكاء الاصطناعي خاطئة؛ تأكد مع خبير.</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr"/>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>HEIC photo: it will be converted to JPEG when you analyse it.</t>
+          <t>JPG, PNG, WebP or HEIC, up to 10 MB</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1131,36 +1131,36 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>HEIC photo: it will be converted to JPEG when you analyse it.</t>
+          <t>JPG, PNG, WebP or HEIC, up to 10 MB</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Hoton HEIC: za a mayar da shi JPEG idan ka fara bincike.</t>
+          <t>JPG, PNG, WebP ko HEIC, har zuwa 10 MB</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Fọ́tò HEIC: a ó yí i padà sí JPEG nígbà tí o bá ṣe àyẹ̀wò.</t>
+          <t>JPG, PNG, WebP tàbí HEIC, títí dé 10 MB</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Foto HEIC: a ga-agbanwe ya ka ọ bụrụ JPEG mgbe ị nyochara ya.</t>
+          <t>JPG, PNG, WebP ma ọ bụ HEIC, ruo 10 MB</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Photo HEIC : elle sera convertie en JPEG lors de l'analyse.</t>
+          <t>JPG, PNG, WebP ou HEIC, jusqu'à 10 Mo</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>صورة HEIC: سيتم تحويلها إلى JPEG عند التحليل.</t>
+          <t>JPG أو PNG أو WebP أو HEIC، حتى 10 ميغابايت</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr"/>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>You have used all :limit scans this month. Upgrade your plan or wait until :date.</t>
+          <t>This file type is not supported. Choose a JPG, PNG, WebP or HEIC photo.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1183,36 +1183,36 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>You have used all :limit scans this month. Upgrade your plan or wait until :date.</t>
+          <t>This file type is not supported. Choose a JPG, PNG, WebP or HEIC photo.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Ka yi amfani da duk binciken :limit na wannan watan. Haɓaka tsarinka ko ka jira har zuwa :date.</t>
+          <t>Ba a karɓar irin wannan fayil ba. Zaɓi hoton JPG, PNG, WebP ko HEIC.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>O ti lo gbogbo àyẹ̀wò :limit rẹ fún oṣù yìí. Ṣe àfikún ètò rẹ tàbí dúró títí di :date.</t>
+          <t>A kò gba irú fáìlì yìí. Yan fọ́tò JPG, PNG, WebP tàbí HEIC.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Ị jirila nyocha :limit niile nke ọnwa a. Kwalite atụmatụ gị ma ọ bụ chere ruo :date.</t>
+          <t>Anaghị anabata ụdị faịlụ a. Họrọ foto JPG, PNG, WebP ma ọ bụ HEIC.</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Vous avez utilisé vos :limit analyses de ce mois. Passez à une offre supérieure ou attendez le :date.</t>
+          <t>Ce type de fichier n'est pas pris en charge. Choisissez une photo JPG, PNG, WebP ou HEIC.</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>لقد استخدمت كل الفحوصات الـ :limit لهذا الشهر. قم بترقية خطتك أو انتظر حتى :date.</t>
+          <t>نوع الملف هذا غير مدعوم. اختر صورة JPG أو PNG أو WebP أو HEIC.</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr"/>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Your login has expired. Please sign in again.</t>
+          <t>HEIC photo: it will be converted to JPEG when you analyse it.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1235,36 +1235,36 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Your login has expired. Please sign in again.</t>
+          <t>HEIC photo: it will be converted to JPEG when you analyse it.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Lokacin shigarka ya ƙare. Don Allah ka sake shiga.</t>
+          <t>Hoton HEIC: za a mayar da shi JPEG idan ka fara bincike.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Ìwọlé rẹ ti parí. Jọ̀wọ́ wọlé lẹ́ẹ̀kan sí i.</t>
+          <t>Fọ́tò HEIC: a ó yí i padà sí JPEG nígbà tí o bá ṣe àyẹ̀wò.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Ntinye gị agwụla. Biko banye ọzọ.</t>
+          <t>Foto HEIC: a ga-agbanwe ya ka ọ bụrụ JPEG mgbe ị nyochara ya.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Votre session a expiré. Veuillez vous reconnecter.</t>
+          <t>Photo HEIC : elle sera convertie en JPEG lors de l'analyse.</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>انتهت صلاحية تسجيل الدخول. يرجى تسجيل الدخول مرة أخرى.</t>
+          <t>صورة HEIC: سيتم تحويلها إلى JPEG عند التحليل.</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>This photo is too large (over 10 MB). Choose a smaller photo or take a new one.</t>
+          <t>You have used all :limit scans this month. Upgrade your plan or wait until :date.</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1287,36 +1287,36 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>This photo is too large (over 10 MB). Choose a smaller photo or take a new one.</t>
+          <t>You have used all :limit scans this month. Upgrade your plan or wait until :date.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Wannan hoton ya yi girma da yawa (sama da 10 MB). Zaɓi ƙaramin hoto ko ka ɗauki sabo.</t>
+          <t>Ka yi amfani da duk binciken :limit na wannan watan. Haɓaka tsarinka ko ka jira har zuwa :date.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Fọ́tò yìí ti tóbi jù (ju 10 MB lọ). Yan fọ́tò kékeré tàbí ya tuntun.</t>
+          <t>O ti lo gbogbo àyẹ̀wò :limit rẹ fún oṣù yìí. Ṣe àfikún ètò rẹ tàbí dúró títí di :date.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Foto a buru oke ibu (karịa 10 MB). Họrọ foto pere mpe ma ọ bụ see nke ọhụrụ.</t>
+          <t>Ị jirila nyocha :limit niile nke ọnwa a. Kwalite atụmatụ gị ma ọ bụ chere ruo :date.</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Cette photo est trop lourde (plus de 10 Mo). Choisissez une photo plus petite ou prenez-en une nouvelle.</t>
+          <t>Vous avez utilisé vos :limit analyses de ce mois. Passez à une offre supérieure ou attendez le :date.</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>هذه الصورة كبيرة جدًا (أكثر من 10 ميغابايت). اختر صورة أصغر أو التقط صورة جديدة.</t>
+          <t>لقد استخدمت كل الفحوصات الـ :limit لهذا الشهر. قم بترقية خطتك أو انتظر حتى :date.</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr"/>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>This file is not a photo we can read. Choose a JPG, PNG, WebP or HEIC photo.</t>
+          <t>Your login has expired. Please sign in again.</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1339,36 +1339,36 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>This file is not a photo we can read. Choose a JPG, PNG, WebP or HEIC photo.</t>
+          <t>Your login has expired. Please sign in again.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Wannan fayil ba hoto ne da za mu iya karantawa ba. Zaɓi hoton JPG, PNG, WebP ko HEIC.</t>
+          <t>Lokacin shigarka ya ƙare. Don Allah ka sake shiga.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Fáìlì yìí kì í ṣe fọ́tò tí a lè kà. Yan fọ́tò JPG, PNG, WebP tàbí HEIC.</t>
+          <t>Ìwọlé rẹ ti parí. Jọ̀wọ́ wọlé lẹ́ẹ̀kan sí i.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Faịlụ a abụghị foto anyị nwere ike ịgụ. Họrọ foto JPG, PNG, WebP ma ọ bụ HEIC.</t>
+          <t>Ntinye gị agwụla. Biko banye ọzọ.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Ce fichier n'est pas une photo lisible. Choisissez une photo JPG, PNG, WebP ou HEIC.</t>
+          <t>Votre session a expiré. Veuillez vous reconnecter.</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>هذا الملف ليس صورة يمكننا قراءتها. اختر صورة JPG أو PNG أو WebP أو HEIC.</t>
+          <t>انتهت صلاحية تسجيل الدخول. يرجى تسجيل الدخول مرة أخرى.</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr"/>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>The photo did not finish uploading. Check your connection and try again.</t>
+          <t>This photo is too large (over 10 MB). Choose a smaller photo or take a new one.</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1391,36 +1391,36 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>The photo did not finish uploading. Check your connection and try again.</t>
+          <t>This photo is too large (over 10 MB). Choose a smaller photo or take a new one.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Hoton bai gama lodawa ba. Duba hanyar sadarwarka ka sake gwadawa.</t>
+          <t>Wannan hoton ya yi girma da yawa (sama da 10 MB). Zaɓi ƙaramin hoto ko ka ɗauki sabo.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Fọ́tò náà kò parí gbígbéjáde. Ṣàyẹ̀wò ìsopọ̀ rẹ kí o sì gbìyànjú lẹ́ẹ̀kan sí i.</t>
+          <t>Fọ́tò yìí ti tóbi jù (ju 10 MB lọ). Yan fọ́tò kékeré tàbí ya tuntun.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Foto ahụ ebugoghị nke ọma. Lelee njikọ gị ma nwaa ọzọ.</t>
+          <t>Foto a buru oke ibu (karịa 10 MB). Họrọ foto pere mpe ma ọ bụ see nke ọhụrụ.</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>La photo n'a pas fini de se télécharger. Vérifiez votre connexion et réessayez.</t>
+          <t>Cette photo est trop lourde (plus de 10 Mo). Choisissez une photo plus petite ou prenez-en une nouvelle.</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>لم يكتمل رفع الصورة. تحقق من اتصالك وحاول مرة أخرى.</t>
+          <t>هذه الصورة كبيرة جدًا (أكثر من 10 ميغابايت). اختر صورة أصغر أو التقط صورة جديدة.</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr"/>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Please check this part of the form: :field.</t>
+          <t>This file is not a photo we can read. Choose a JPG, PNG, WebP or HEIC photo.</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1443,36 +1443,36 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Please check this part of the form: :field.</t>
+          <t>This file is not a photo we can read. Choose a JPG, PNG, WebP or HEIC photo.</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Don Allah duba wannan sashe na fom: :field.</t>
+          <t>Wannan fayil ba hoto ne da za mu iya karantawa ba. Zaɓi hoton JPG, PNG, WebP ko HEIC.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Jọ̀wọ́ ṣàyẹ̀wò apá yìí nínú fọ́ọ̀mù náà: :field.</t>
+          <t>Fáìlì yìí kì í ṣe fọ́tò tí a lè kà. Yan fọ́tò JPG, PNG, WebP tàbí HEIC.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Biko lelee akụkụ a nke fọm ahụ: :field.</t>
+          <t>Faịlụ a abụghị foto anyị nwere ike ịgụ. Họrọ foto JPG, PNG, WebP ma ọ bụ HEIC.</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Veuillez vérifier cette partie du formulaire : :field.</t>
+          <t>Ce fichier n'est pas une photo lisible. Choisissez une photo JPG, PNG, WebP ou HEIC.</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>يرجى التحقق من هذا الجزء من النموذج: :field.</t>
+          <t>هذا الملف ليس صورة يمكننا قراءتها. اختر صورة JPG أو PNG أو WebP أو HEIC.</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr"/>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>You are sending scans too quickly. Wait a minute, then try again.</t>
+          <t>The photo did not finish uploading. Check your connection and try again.</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1495,36 +1495,36 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>You are sending scans too quickly. Wait a minute, then try again.</t>
+          <t>The photo did not finish uploading. Check your connection and try again.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Kana aika bincike da sauri sosai. Jira minti ɗaya, sannan ka sake gwadawa.</t>
+          <t>Hoton bai gama lodawa ba. Duba hanyar sadarwarka ka sake gwadawa.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>O ń fi àyẹ̀wò ránṣẹ́ ní kíákíá jù. Dúró fún ìṣẹ́jú kan, lẹ́yìn náà gbìyànjú lẹ́ẹ̀kan sí i.</t>
+          <t>Fọ́tò náà kò parí gbígbéjáde. Ṣàyẹ̀wò ìsopọ̀ rẹ kí o sì gbìyànjú lẹ́ẹ̀kan sí i.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Ị na-eziga nyocha ngwa ngwa. Chere otu nkeji, wee nwaa ọzọ.</t>
+          <t>Foto ahụ ebugoghị nke ọma. Lelee njikọ gị ma nwaa ọzọ.</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Vous envoyez des analyses trop rapidement. Attendez une minute, puis réessayez.</t>
+          <t>La photo n'a pas fini de se télécharger. Vérifiez votre connexion et réessayez.</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>أنت ترسل الفحوصات بسرعة كبيرة. انتظر دقيقة ثم حاول مرة أخرى.</t>
+          <t>لم يكتمل رفع الصورة. تحقق من اتصالك وحاول مرة أخرى.</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr"/>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+          <t>Please check this part of the form: :field.</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1547,36 +1547,36 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+          <t>Please check this part of the form: :field.</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+          <t>Don Allah duba wannan sashe na fom: :field.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+          <t>Jọ̀wọ́ ṣàyẹ̀wò apá yìí nínú fọ́ọ̀mù náà: :field.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+          <t>Biko lelee akụkụ a nke fọm ahụ: :field.</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+          <t>Veuillez vérifier cette partie du formulaire : :field.</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>خدمة التحليل لدينا غير متاحة مؤقتًا. لم يتم احتساب فحصك. يرجى المحاولة مرة أخرى بعد بضع دقائق.</t>
+          <t>يرجى التحقق من هذا الجزء من النموذج: :field.</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr"/>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>We could not assess this photo. See the tips below and retake it.</t>
+          <t>You are sending scans too quickly. Wait a minute, then try again.</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1599,36 +1599,36 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>We could not assess this photo. See the tips below and retake it.</t>
+          <t>You are sending scans too quickly. Wait a minute, then try again.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Ba mu iya tantance wannan hoton ba. Duba shawarwarin da ke ƙasa ka sake ɗauka.</t>
+          <t>Kana aika bincike da sauri sosai. Jira minti ɗaya, sannan ka sake gwadawa.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>A kò lè ṣàyẹ̀wò fọ́tò yìí. Wo àwọn ìmọ̀ràn ní ìsàlẹ̀ kí o sì tún ya á.</t>
+          <t>O ń fi àyẹ̀wò ránṣẹ́ ní kíákíá jù. Dúró fún ìṣẹ́jú kan, lẹ́yìn náà gbìyànjú lẹ́ẹ̀kan sí i.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Anyị enweghị ike inyocha foto a. Lee ndụmọdụ dị n'okpuru ma see ya ọzọ.</t>
+          <t>Ị na-eziga nyocha ngwa ngwa. Chere otu nkeji, wee nwaa ọzọ.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Nous n'avons pas pu évaluer cette photo. Consultez les conseils ci-dessous et reprenez-la.</t>
+          <t>Vous envoyez des analyses trop rapidement. Attendez une minute, puis réessayez.</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>لم نتمكن من تقييم هذه الصورة. راجع النصائح أدناه وأعد التقاطها.</t>
+          <t>أنت ترسل الفحوصات بسرعة كبيرة. انتظر دقيقة ثم حاول مرة أخرى.</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr"/>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Something went wrong on our side. Your scan was NOT counted. Please try again, and contact support with the reference below if it keeps happening.</t>
+          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1651,36 +1651,36 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Something went wrong on our side. Your scan was NOT counted. Please try again, and contact support with the reference below if it keeps happening.</t>
+          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Wani abu ya lalace a ɓangarenmu. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa, kuma ka tuntuɓi tallafi da lambar shaida da ke ƙasa idan ya ci gaba.</t>
+          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Nǹkan kan ṣẹlẹ̀ ní ẹ̀gbẹ́ wa. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i, kí o sì kàn sí ìrànlọ́wọ́ pẹ̀lú ìtọ́kasí ní ìsàlẹ̀ tí ó bá ń ṣẹlẹ̀ síbẹ̀.</t>
+          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Ihe ọjọọ mere n'akụkụ anyị. A GỤGHỊ nyocha gị. Biko nwaa ọzọ, kpọtụrụ ndị nkwado jiri ntụaka dị n'okpuru ma ọ bụrụ na ọ na-eme ọzọ.</t>
+          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Un problème est survenu de notre côté. Votre analyse n'a PAS été comptée. Veuillez réessayer et contactez l'assistance avec la référence ci-dessous si le problème persiste.</t>
+          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>حدث خطأ من جانبنا. لم يتم احتساب فحصك. يرجى المحاولة مرة أخرى، وتواصل مع الدعم مع ذكر المرجع أدناه إذا تكرر الأمر.</t>
+          <t>خدمة التحليل لدينا غير متاحة مؤقتًا. لم يتم احتساب فحصك. يرجى المحاولة مرة أخرى بعد بضع دقائق.</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr"/>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Reference: :ref</t>
+          <t>We could not assess this photo. See the tips below and retake it.</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1703,36 +1703,36 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Reference: :ref</t>
+          <t>We could not assess this photo. See the tips below and retake it.</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Lambar shaida: :ref</t>
+          <t>Ba mu iya tantance wannan hoton ba. Duba shawarwarin da ke ƙasa ka sake ɗauka.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Ìtọ́kasí: :ref</t>
+          <t>A kò lè ṣàyẹ̀wò fọ́tò yìí. Wo àwọn ìmọ̀ràn ní ìsàlẹ̀ kí o sì tún ya á.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Ntụaka: :ref</t>
+          <t>Anyị enweghị ike inyocha foto a. Lee ndụmọdụ dị n'okpuru ma see ya ọzọ.</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Référence : :ref</t>
+          <t>Nous n'avons pas pu évaluer cette photo. Consultez les conseils ci-dessous et reprenez-la.</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>المرجع: :ref</t>
+          <t>لم نتمكن من تقييم هذه الصورة. راجع النصائح أدناه وأعد التقاطها.</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr"/>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Reference:</t>
+          <t>Something went wrong on our side. Your scan was NOT counted. Please try again, and contact support with the reference below if it keeps happening.</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1755,36 +1755,36 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Reference:</t>
+          <t>Something went wrong on our side. Your scan was NOT counted. Please try again, and contact support with the reference below if it keeps happening.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Lambar shaida:</t>
+          <t>Wani abu ya lalace a ɓangarenmu. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa, kuma ka tuntuɓi tallafi da lambar shaida da ke ƙasa idan ya ci gaba.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Ìtọ́kasí:</t>
+          <t>Nǹkan kan ṣẹlẹ̀ ní ẹ̀gbẹ́ wa. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i, kí o sì kàn sí ìrànlọ́wọ́ pẹ̀lú ìtọ́kasí ní ìsàlẹ̀ tí ó bá ń ṣẹlẹ̀ síbẹ̀.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Ntụaka:</t>
+          <t>Ihe ọjọọ mere n'akụkụ anyị. A GỤGHỊ nyocha gị. Biko nwaa ọzọ, kpọtụrụ ndị nkwado jiri ntụaka dị n'okpuru ma ọ bụrụ na ọ na-eme ọzọ.</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Référence :</t>
+          <t>Un problème est survenu de notre côté. Votre analyse n'a PAS été comptée. Veuillez réessayer et contactez l'assistance avec la référence ci-dessous si le problème persiste.</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr"/>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>المرجع:</t>
+          <t>حدث خطأ من جانبنا. لم يتم احتساب فحصك. يرجى المحاولة مرة أخرى، وتواصل مع الدعم مع ذكر المرجع أدناه إذا تكرر الأمر.</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr"/>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>the photo</t>
+          <t>Reference: :ref</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1807,36 +1807,36 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>the photo</t>
+          <t>Reference: :ref</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>hoton</t>
+          <t>Lambar shaida: :ref</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>fọ́tò náà</t>
+          <t>Ìtọ́kasí: :ref</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>foto ahụ</t>
+          <t>Ntụaka: :ref</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>la photo</t>
+          <t>Référence : :ref</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr"/>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>الصورة</t>
+          <t>المرجع: :ref</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>what you are scanning</t>
+          <t>Reference:</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1859,36 +1859,36 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>what you are scanning</t>
+          <t>Reference:</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>abin da kake bincika</t>
+          <t>Lambar shaida:</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>ohun tí o ń ṣàyẹ̀wò</t>
+          <t>Ìtọ́kasí:</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>ihe ị na-enyocha</t>
+          <t>Ntụaka:</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>ce que vous analysez</t>
+          <t>Référence :</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>ما تقوم بفحصه</t>
+          <t>المرجع:</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr"/>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>the animal type</t>
+          <t>the photo</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1911,36 +1911,36 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>the animal type</t>
+          <t>the photo</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>nau'in dabba</t>
+          <t>hoton</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>irú ẹranko</t>
+          <t>fọ́tò náà</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>ụdị anụmanụ</t>
+          <t>foto ahụ</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>le type d'animal</t>
+          <t>la photo</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>نوع الحيوان</t>
+          <t>الصورة</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr"/>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>the assessment type</t>
+          <t>what you are scanning</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1963,36 +1963,36 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>the assessment type</t>
+          <t>what you are scanning</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>nau'in bincike</t>
+          <t>abin da kake bincika</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>irú àyẹ̀wò</t>
+          <t>ohun tí o ń ṣàyẹ̀wò</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>ụdị nyocha</t>
+          <t>ihe ị na-enyocha</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr"/>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>le type d'évaluation</t>
+          <t>ce que vous analysez</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr"/>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>نوع التقييم</t>
+          <t>ما تقوم بفحصه</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr"/>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>the crop details</t>
+          <t>the animal type</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -2015,36 +2015,36 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>the crop details</t>
+          <t>the animal type</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>bayanan amfanin gona</t>
+          <t>nau'in dabba</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>àlàyé irúgbìn</t>
+          <t>irú ẹranko</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>nkọwa ihe ọkụkụ</t>
+          <t>ụdị anụmanụ</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>les détails de la culture</t>
+          <t>le type d'animal</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>تفاصيل المحصول</t>
+          <t>نوع الحيوان</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr"/>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>the location</t>
+          <t>the assessment type</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2067,36 +2067,36 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>the location</t>
+          <t>the assessment type</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>wurin</t>
+          <t>nau'in bincike</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>ibi náà</t>
+          <t>irú àyẹ̀wò</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>ebe ahụ</t>
+          <t>ụdị nyocha</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr"/>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>le lieu</t>
+          <t>le type d'évaluation</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr"/>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>الموقع</t>
+          <t>نوع التقييم</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr"/>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>the form</t>
+          <t>the crop details</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2119,36 +2119,36 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>the form</t>
+          <t>the crop details</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>fom ɗin</t>
+          <t>bayanan amfanin gona</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>fọ́ọ̀mù náà</t>
+          <t>àlàyé irúgbìn</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>fọm ahụ</t>
+          <t>nkọwa ihe ọkụkụ</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>le formulaire</t>
+          <t>les détails de la culture</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr"/>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>النموذج</t>
+          <t>تفاصيل المحصول</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr"/>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Try again</t>
+          <t>the location</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2171,36 +2171,36 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Try again</t>
+          <t>the location</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Sake gwadawa</t>
+          <t>wurin</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Gbìyànjú lẹ́ẹ̀kan sí i</t>
+          <t>ibi náà</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Nwaa ọzọ</t>
+          <t>ebe ahụ</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Réessayer</t>
+          <t>le lieu</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr"/>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>حاول مرة أخرى</t>
+          <t>الموقع</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr"/>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Sign in</t>
+          <t>the form</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2223,36 +2223,36 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Sign in</t>
+          <t>the form</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Shiga</t>
+          <t>fom ɗin</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Wọlé</t>
+          <t>fọ́ọ̀mù náà</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Banye</t>
+          <t>fọm ahụ</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Se connecter</t>
+          <t>le formulaire</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr"/>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>تسجيل الدخول</t>
+          <t>النموذج</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr"/>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Upgrade plan</t>
+          <t>Try again</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2275,36 +2275,36 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Upgrade plan</t>
+          <t>Try again</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Haɓaka tsari</t>
+          <t>Sake gwadawa</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Ṣe àfikún ètò</t>
+          <t>Gbìyànjú lẹ́ẹ̀kan sí i</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Kwalite atụmatụ</t>
+          <t>Nwaa ọzọ</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Changer d'offre</t>
+          <t>Réessayer</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr"/>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>ترقية الخطة</t>
+          <t>حاول مرة أخرى</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr"/>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Choose another photo</t>
+          <t>Sign in</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2327,36 +2327,36 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Choose another photo</t>
+          <t>Sign in</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Zaɓi wani hoto</t>
+          <t>Shiga</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Yan fọ́tò mìíràn</t>
+          <t>Wọlé</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Họrọ foto ọzọ</t>
+          <t>Banye</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr"/>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Choisir une autre photo</t>
+          <t>Se connecter</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr"/>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>اختر صورة أخرى</t>
+          <t>تسجيل الدخول</t>
         </is>
       </c>
       <c r="N35" s="4" t="inlineStr"/>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>This scan did not complete</t>
+          <t>Upgrade plan</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2379,36 +2379,36 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>This scan did not complete</t>
+          <t>Upgrade plan</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Wannan binciken bai kammala ba</t>
+          <t>Haɓaka tsari</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Àyẹ̀wò yìí kò parí</t>
+          <t>Ṣe àfikún ètò</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Nyocha a emechaghị</t>
+          <t>Kwalite atụmatụ</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr"/>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Cette analyse n'a pas abouti</t>
+          <t>Changer d'offre</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr"/>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t>لم يكتمل هذا الفحص</t>
+          <t>ترقية الخطة</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr"/>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service was unavailable, so there is no result and this scan was not counted. Please scan again.</t>
+          <t>Choose another photo</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2431,36 +2431,36 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service was unavailable, so there is no result and this scan was not counted. Please scan again.</t>
+          <t>Choose another photo</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Sabis ɗin bincikenmu ba ya aiki, don haka babu sakamako kuma ba a ƙirga wannan binciken ba. Don Allah ka sake bincike.</t>
+          <t>Zaɓi wani hoto</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Iṣẹ́ àyẹ̀wò wa kò sí, nítorí náà kò sí èsì, a kò sì ka àyẹ̀wò yìí. Jọ̀wọ́ ṣàyẹ̀wò lẹ́ẹ̀kan sí i.</t>
+          <t>Yan fọ́tò mìíràn</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Ọrụ nyocha anyị adịghị, ya mere enweghị nsonaazụ, a gụghịkwa nyocha a. Biko nyochaa ọzọ.</t>
+          <t>Họrọ foto ọzọ</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Notre service d'analyse était indisponible : il n'y a pas de résultat et cette analyse n'a pas été comptée. Veuillez refaire l'analyse.</t>
+          <t>Choisir une autre photo</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t>كانت خدمة التحليل لدينا غير متاحة، لذلك لا توجد نتيجة ولم يتم احتساب هذا الفحص. يرجى الفحص مرة أخرى.</t>
+          <t>اختر صورة أخرى</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr"/>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>No result: this scan did not complete</t>
+          <t>This scan did not complete</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2483,36 +2483,36 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>No result: this scan did not complete</t>
+          <t>This scan did not complete</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Babu sakamako: wannan binciken bai kammala ba</t>
+          <t>Wannan binciken bai kammala ba</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Kò sí èsì: àyẹ̀wò yìí kò parí</t>
+          <t>Àyẹ̀wò yìí kò parí</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Enweghị nsonaazụ: nyocha a emechaghị</t>
+          <t>Nyocha a emechaghị</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Aucun résultat : cette analyse n'a pas abouti</t>
+          <t>Cette analyse n'a pas abouti</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr"/>
       <c r="M38" s="3" t="inlineStr">
         <is>
-          <t>لا توجد نتيجة: لم يكتمل هذا الفحص</t>
+          <t>لم يكتمل هذا الفحص</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr"/>
@@ -2520,12 +2520,12 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>web</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>soilScanDesc</t>
+          <t>Our analysis service was unavailable, so there is no result and this scan was not counted. Please scan again.</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2535,53 +2535,49 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Nutrients &amp; recommendations</t>
+          <t>Our analysis service was unavailable, so there is no result and this scan was not counted. Please scan again.</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Abinci da shawarwari</t>
+          <t>Sabis ɗin bincikenmu ba ya aiki, don haka babu sakamako kuma ba a ƙirga wannan binciken ba. Don Allah ka sake bincike.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Àwọn èròjà ilẹ̀ àti ìmọ̀ràn</t>
+          <t>Iṣẹ́ àyẹ̀wò wa kò sí, nítorí náà kò sí èsì, a kò sì ka àyẹ̀wò yìí. Jọ̀wọ́ ṣàyẹ̀wò lẹ́ẹ̀kan sí i.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Nri ala na ndụmọdụ</t>
+          <t>Ọrụ nyocha anyị adịghị, ya mere enweghị nsonaazụ, a gụghịkwa nyocha a. Biko nyochaa ọzọ.</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr"/>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Nutriments et recommandations</t>
+          <t>Notre service d'analyse était indisponible : il n'y a pas de résultat et cette analyse n'a pas été comptée. Veuillez refaire l'analyse.</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t>(not in the app)</t>
-        </is>
-      </c>
-      <c r="N39" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
+          <t>كانت خدمة التحليل لدينا غير متاحة، لذلك لا توجد نتيجة ولم يتم احتساب هذا الفحص. يرجى الفحص مرة أخرى.</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>web</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>notCertain</t>
+          <t>No result: this scan did not complete</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2591,43 +2587,39 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Not certain</t>
+          <t>No result: this scan did not complete</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Ba a tabbata ba</t>
+          <t>Babu sakamako: wannan binciken bai kammala ba</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Kò dájú</t>
+          <t>Kò sí èsì: àyẹ̀wò yìí kò parí</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>O doghị anya</t>
+          <t>Enweghị nsonaazụ: nyocha a emechaghị</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr"/>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Pas certain</t>
+          <t>Aucun résultat : cette analyse n'a pas abouti</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr"/>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>(not in the app)</t>
-        </is>
-      </c>
-      <c r="N40" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
+          <t>لا توجد نتيجة: لم يكتمل هذا الفحص</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2637,7 +2629,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>notCertainBody</t>
+          <t>soilScanDesc</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2647,30 +2639,30 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>The AI is not sure enough to give one diagnosis. These are the possible conditions:</t>
+          <t>Nutrients &amp; recommendations</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>AI ba ta da isasshen tabbaci don ba da cuta ɗaya. Ga cututtukan da za su iya kasancewa:</t>
+          <t>Abinci da shawarwari</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>AI kò ní ìdánilójú tó láti fún ọ ní àrùn kan ṣoṣo. Àwọn àrùn tó ṣeé ṣe nìwọ̀nyí:</t>
+          <t>Àwọn èròjà ilẹ̀ àti ìmọ̀ràn</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>AI enweghị ezigbo ntụkwasị obi iji kwuo otu ọrịa. Ndị a bụ ọrịa ndị nwere ike ịbụ:</t>
+          <t>Nri ala na ndụmọdụ</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>L'IA n'est pas assez sûre pour donner un seul diagnostic. Voici les problèmes possibles :</t>
+          <t>Nutriments et recommandations</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr"/>
@@ -2693,7 +2685,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>possibleConditions</t>
+          <t>notCertain</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2703,30 +2695,30 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Possible conditions</t>
+          <t>Not certain</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Cututtukan da za su iya kasancewa</t>
+          <t>Ba a tabbata ba</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Àwọn àrùn tó ṣeé ṣe</t>
+          <t>Kò dájú</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Ọrịa ndị nwere ike ịbụ</t>
+          <t>O doghị anya</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Problèmes possibles</t>
+          <t>Pas certain</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr"/>
@@ -2749,7 +2741,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>confirmWithExpert</t>
+          <t>notCertainBody</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2759,30 +2751,30 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Please confirm with a vet or extension officer before treating.</t>
+          <t>The AI is not sure enough to give one diagnosis. These are the possible conditions:</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
+          <t>AI ba ta da isasshen tabbaci don ba da cuta ɗaya. Ga cututtukan da za su iya kasancewa:</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Jọ̀wọ́ fìdí rẹ̀ múlẹ̀ pẹ̀lú dókítà ẹranko tàbí òṣìṣẹ́ àgbẹ̀ kí o tó tọ́jú.</t>
+          <t>AI kò ní ìdánilójú tó láti fún ọ ní àrùn kan ṣoṣo. Àwọn àrùn tó ṣeé ṣe nìwọ̀nyí:</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Biko kwado ya na dọkịta anụmanụ ma ọ bụ onye ndụmọdụ ugbo tupu ị gwọọ.</t>
+          <t>AI enweghị ezigbo ntụkwasị obi iji kwuo otu ọrịa. Ndị a bụ ọrịa ndị nwere ike ịbụ:</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
+          <t>L'IA n'est pas assez sûre pour donner un seul diagnostic. Voici les problèmes possibles :</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr"/>
@@ -2805,7 +2797,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>urgency</t>
+          <t>possibleConditions</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2815,30 +2807,30 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Urgency</t>
+          <t>Possible conditions</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Gaggawa</t>
+          <t>Cututtukan da za su iya kasancewa</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>Àwọn àrùn tó ṣeé ṣe</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>Ọrịa ndị nwere ike ịbụ</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Urgence</t>
+          <t>Problèmes possibles</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr"/>
@@ -2861,7 +2853,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>likely</t>
+          <t>confirmWithExpert</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2871,30 +2863,30 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Likely</t>
+          <t>Please confirm with a vet or extension officer before treating.</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Wataƙila</t>
+          <t>Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr"/>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>Jọ̀wọ́ fìdí rẹ̀ múlẹ̀ pẹ̀lú dókítà ẹranko tàbí òṣìṣẹ́ àgbẹ̀ kí o tó tọ́jú.</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>Biko kwado ya na dọkịta anụmanụ ma ọ bụ onye ndụmọdụ ugbo tupu ị gwọọ.</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Probable</t>
+          <t>Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr"/>
@@ -2917,7 +2909,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>likelyConfirm</t>
+          <t>urgency</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2927,12 +2919,12 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>The AI thinks this is likely, but is not fully sure. Please confirm with a vet or extension officer before treating.</t>
+          <t>Urgency</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>AI na ganin hakan ne mai yiwuwa, amma bai tabbata sosai ba. Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
+          <t>Gaggawa</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -2950,7 +2942,7 @@
       <c r="J46" s="4" t="inlineStr"/>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>L'IA pense que c'est probable, mais n'en est pas tout à fait sûre. Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
+          <t>Urgence</t>
         </is>
       </c>
       <c r="L46" s="4" t="inlineStr"/>
@@ -2973,7 +2965,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>aiDisclaimer</t>
+          <t>likely</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2983,30 +2975,30 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>AI guidance can be wrong; confirm with an expert.</t>
+          <t>Likely</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Shawarar AI na iya yin kuskure; ka tabbatar da ƙwararre.</t>
+          <t>Wataƙila</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr"/>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Ìmọ̀ràn AI lè ṣàṣìṣe; fìdí rẹ̀ múlẹ̀ pẹ̀lú amòye.</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Ndụmọdụ AI nwere ike ihie ụzọ; kwado ya na ọkachamara.</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr"/>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Les conseils de l'IA peuvent être erronés ; confirmez auprès d'un expert.</t>
+          <t>Probable</t>
         </is>
       </c>
       <c r="L47" s="4" t="inlineStr"/>
@@ -3024,12 +3016,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>app-errors</t>
+          <t>app</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>likelyConfirm</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -3039,30 +3031,30 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Scan not completed</t>
+          <t>The AI thinks this is likely, but is not fully sure. Please confirm with a vet or extension officer before treating.</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Binciken bai kammala ba</t>
+          <t>AI na ganin hakan ne mai yiwuwa, amma bai tabbata sosai ba. Don Allah ka tabbatar da likitan dabbobi ko jami'in faɗakarwa kafin ka yi magani.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr"/>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Àyẹ̀wò kò parí</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Nyocha emechaghị</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr"/>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Analyse non terminée</t>
+          <t>L'IA pense que c'est probable, mais n'en est pas tout à fait sûre. Veuillez confirmer avec un vétérinaire ou un agent de vulgarisation avant de traiter.</t>
         </is>
       </c>
       <c r="L48" s="4" t="inlineStr"/>
@@ -3080,12 +3072,12 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>app-errors</t>
+          <t>app</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>aiDisclaimer</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -3095,30 +3087,30 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>AI guidance can be wrong; confirm with an expert.</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Lambar shaida</t>
+          <t>Shawarar AI na iya yin kuskure; ka tabbatar da ƙwararre.</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr"/>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Ìtọ́kasí</t>
+          <t>Ìmọ̀ràn AI lè ṣàṣìṣe; fìdí rẹ̀ múlẹ̀ pẹ̀lú amòye.</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Ntụaka</t>
+          <t>Ndụmọdụ AI nwere ike ihie ụzọ; kwado ya na ọkachamara.</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr"/>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Référence</t>
+          <t>Les conseils de l'IA peuvent être erronés ; confirmez auprès d'un expert.</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr"/>
@@ -3141,7 +3133,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>retry</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3151,30 +3143,30 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Try again</t>
+          <t>Scan not completed</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Sake gwadawa</t>
+          <t>Binciken bai kammala ba</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr"/>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Gbìyànjú lẹ́ẹ̀kan sí i</t>
+          <t>Àyẹ̀wò kò parí</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr"/>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Nwaa ọzọ</t>
+          <t>Nyocha emechaghị</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr"/>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Réessayer</t>
+          <t>Analyse non terminée</t>
         </is>
       </c>
       <c r="L50" s="4" t="inlineStr"/>
@@ -3197,7 +3189,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>signIn</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3207,30 +3199,30 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Sign in</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Shiga</t>
+          <t>Lambar shaida</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr"/>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Wọlé</t>
+          <t>Ìtọ́kasí</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Banye</t>
+          <t>Ntụaka</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr"/>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Se connecter</t>
+          <t>Référence</t>
         </is>
       </c>
       <c r="L51" s="4" t="inlineStr"/>
@@ -3253,7 +3245,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>retry</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3263,30 +3255,30 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Upgrade plan</t>
+          <t>Try again</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Haɓaka tsari</t>
+          <t>Sake gwadawa</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr"/>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Ṣe àfikún ètò</t>
+          <t>Gbìyànjú lẹ́ẹ̀kan sí i</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Kwalite atụmatụ</t>
+          <t>Nwaa ọzọ</t>
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr"/>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Changer d'offre</t>
+          <t>Réessayer</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr"/>
@@ -3309,7 +3301,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>choosePhoto</t>
+          <t>signIn</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -3319,30 +3311,30 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Choose another photo</t>
+          <t>Sign in</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Zaɓi wani hoto</t>
+          <t>Shiga</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr"/>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Yan fọ́tò mìíràn</t>
+          <t>Wọlé</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Họrọ foto ọzọ</t>
+          <t>Banye</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Choisir une autre photo</t>
+          <t>Se connecter</t>
         </is>
       </c>
       <c r="L53" s="4" t="inlineStr"/>
@@ -3365,7 +3357,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>close</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -3375,30 +3367,30 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Upgrade plan</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Rufe</t>
+          <t>Haɓaka tsari</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr"/>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Pa á dé</t>
+          <t>Ṣe àfikún ètò</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Mechie</t>
+          <t>Kwalite atụmatụ</t>
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr"/>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Fermer</t>
+          <t>Changer d'offre</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr"/>
@@ -3421,7 +3413,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>codes.SESSION_EXPIRED</t>
+          <t>choosePhoto</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -3431,30 +3423,30 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Your login has expired. Please sign in again.</t>
+          <t>Choose another photo</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Lokacin shigarka ya ƙare. Don Allah ka sake shiga.</t>
+          <t>Zaɓi wani hoto</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr"/>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Ìwọlé rẹ ti parí. Jọ̀wọ́ wọlé lẹ́ẹ̀kan sí i.</t>
+          <t>Yan fọ́tò mìíràn</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Ntinye gị agwụla. Biko banye ọzọ.</t>
+          <t>Họrọ foto ọzọ</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr"/>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>Votre session a expiré. Veuillez vous reconnecter.</t>
+          <t>Choisir une autre photo</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr"/>
@@ -3477,7 +3469,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>codes.UPLOAD_TOO_LARGE</t>
+          <t>close</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -3487,30 +3479,30 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>This photo is too large (over 10 MB). Choose a smaller photo or take a new one.</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Wannan hoton ya yi girma da yawa (sama da 10 MB). Zaɓi ƙaramin hoto ko ka ɗauki sabo.</t>
+          <t>Rufe</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr"/>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Fọ́tò yìí ti tóbi jù (ju 10 MB lọ). Yan fọ́tò kékeré tàbí ya tuntun.</t>
+          <t>Pa á dé</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr"/>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Foto a buru oke ibu (karịa 10 MB). Họrọ foto pere mpe ma ọ bụ see nke ọhụrụ.</t>
+          <t>Mechie</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr"/>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Cette photo est trop lourde (plus de 10 Mo). Choisissez une photo plus petite ou prenez-en une nouvelle.</t>
+          <t>Fermer</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr"/>
@@ -3533,7 +3525,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>codes.UPLOAD_BAD_FORMAT</t>
+          <t>copy</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -3543,30 +3535,30 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>This file is not a photo we can read. Choose a JPG, PNG, WebP or HEIC photo.</t>
+          <t>Copy details</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Wannan fayil ba hoto ne da za mu iya karantawa ba. Zaɓi hoton JPG, PNG, WebP ko HEIC.</t>
+          <t>Kwafa bayanai</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr"/>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Fáìlì yìí kì í ṣe fọ́tò tí a lè kà. Yan fọ́tò JPG, PNG, WebP tàbí HEIC.</t>
+          <t>Daakọ àlàyé</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr"/>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Faịlụ a abụghị foto anyị nwere ike ịgụ. Họrọ foto JPG, PNG, WebP ma ọ bụ HEIC.</t>
+          <t>Detuo nkọwa</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr"/>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Ce fichier n'est pas une photo lisible. Choisissez une photo JPG, PNG, WebP ou HEIC.</t>
+          <t>Copier les détails</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr"/>
@@ -3589,7 +3581,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>codes.UPLOAD_INTERRUPTED</t>
+          <t>copied</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -3599,30 +3591,30 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>The photo did not finish uploading. Check your connection and try again.</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Hoton bai gama lodawa ba. Duba hanyar sadarwarka ka sake gwadawa.</t>
+          <t>An kwafa</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr"/>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>Fọ́tò náà kò parí gbígbéjáde. Ṣàyẹ̀wò ìsopọ̀ rẹ kí o sì gbìyànjú lẹ́ẹ̀kan sí i.</t>
+          <t>A ti daakọ</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr"/>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Foto ahụ ebugoghị nke ọma. Lelee njikọ gị ma nwaa ọzọ.</t>
+          <t>Edetuola</t>
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr"/>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>La photo n'a pas fini de se télécharger. Vérifiez votre connexion et réessayez.</t>
+          <t>Copié</t>
         </is>
       </c>
       <c r="L58" s="4" t="inlineStr"/>
@@ -3645,7 +3637,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>codes.TOO_MANY_SCANS</t>
+          <t>codes.SESSION_EXPIRED</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3655,30 +3647,30 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>You are sending scans too quickly. Wait a minute, then try again.</t>
+          <t>Your login has expired. Please sign in again.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Kana aika bincike da sauri sosai. Jira minti ɗaya, sannan ka sake gwadawa.</t>
+          <t>Lokacin shigarka ya ƙare. Don Allah ka sake shiga.</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr"/>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>O ń fi àyẹ̀wò ránṣẹ́ ní kíákíá jù. Dúró fún ìṣẹ́jú kan, lẹ́yìn náà gbìyànjú lẹ́ẹ̀kan sí i.</t>
+          <t>Ìwọlé rẹ ti parí. Jọ̀wọ́ wọlé lẹ́ẹ̀kan sí i.</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Ị na-eziga nyocha ngwa ngwa. Chere otu nkeji, wee nwaa ọzọ.</t>
+          <t>Ntinye gị agwụla. Biko banye ọzọ.</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr"/>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Vous envoyez des analyses trop rapidement. Attendez une minute, puis réessayez.</t>
+          <t>Votre session a expiré. Veuillez vous reconnecter.</t>
         </is>
       </c>
       <c r="L59" s="4" t="inlineStr"/>
@@ -3701,7 +3693,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>codes.INTERNAL_ERROR</t>
+          <t>codes.UPLOAD_TOO_LARGE</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -3711,30 +3703,30 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Something went wrong on our side. Your scan was NOT counted. Please try again, and contact support with the reference below if it keeps happening.</t>
+          <t>This photo is too large (over 10 MB). Choose a smaller photo or take a new one.</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Wani abu ya lalace a ɓangarenmu. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa, kuma ka tuntuɓi tallafi da lambar shaida da ke ƙasa idan ya ci gaba.</t>
+          <t>Wannan hoton ya yi girma da yawa (sama da 10 MB). Zaɓi ƙaramin hoto ko ka ɗauki sabo.</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr"/>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Nǹkan kan ṣẹlẹ̀ ní ẹ̀gbẹ́ wa. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i, kí o sì kàn sí ìrànlọ́wọ́ pẹ̀lú ìtọ́kasí ní ìsàlẹ̀ tí ó bá ń ṣẹlẹ̀ síbẹ̀.</t>
+          <t>Fọ́tò yìí ti tóbi jù (ju 10 MB lọ). Yan fọ́tò kékeré tàbí ya tuntun.</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr"/>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>Ihe ọjọọ mere n'akụkụ anyị. A GỤGHỊ nyocha gị. Biko nwaa ọzọ, kpọtụrụ ndị nkwado jiri ntụaka dị n'okpuru ma ọ bụrụ na ọ na-eme ọzọ.</t>
+          <t>Foto a buru oke ibu (karịa 10 MB). Họrọ foto pere mpe ma ọ bụ see nke ọhụrụ.</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr"/>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Un problème est survenu de notre côté. Votre analyse n'a PAS été comptée. Veuillez réessayer et contactez l'assistance avec la référence ci-dessous si le problème persiste.</t>
+          <t>Cette photo est trop lourde (plus de 10 Mo). Choisissez une photo plus petite ou prenez-en une nouvelle.</t>
         </is>
       </c>
       <c r="L60" s="4" t="inlineStr"/>
@@ -3757,7 +3749,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>codes.ENGINE_UNREACHABLE</t>
+          <t>codes.UPLOAD_BAD_FORMAT</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -3767,30 +3759,30 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+          <t>This file is not a photo we can read. Choose a JPG, PNG, WebP or HEIC photo.</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+          <t>Wannan fayil ba hoto ne da za mu iya karantawa ba. Zaɓi hoton JPG, PNG, WebP ko HEIC.</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr"/>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+          <t>Fáìlì yìí kì í ṣe fọ́tò tí a lè kà. Yan fọ́tò JPG, PNG, WebP tàbí HEIC.</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+          <t>Faịlụ a abụghị foto anyị nwere ike ịgụ. Họrọ foto JPG, PNG, WebP ma ọ bụ HEIC.</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr"/>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+          <t>Ce fichier n'est pas une photo lisible. Choisissez une photo JPG, PNG, WebP ou HEIC.</t>
         </is>
       </c>
       <c r="L61" s="4" t="inlineStr"/>
@@ -3813,7 +3805,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>codes.ENGINE_AUTH_FAILED</t>
+          <t>codes.UPLOAD_INTERRUPTED</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -3823,30 +3815,30 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+          <t>The photo did not finish uploading. Check your connection and try again.</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+          <t>Hoton bai gama lodawa ba. Duba hanyar sadarwarka ka sake gwadawa.</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr"/>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+          <t>Fọ́tò náà kò parí gbígbéjáde. Ṣàyẹ̀wò ìsopọ̀ rẹ kí o sì gbìyànjú lẹ́ẹ̀kan sí i.</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+          <t>Foto ahụ ebugoghị nke ọma. Lelee njikọ gị ma nwaa ọzọ.</t>
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr"/>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+          <t>La photo n'a pas fini de se télécharger. Vérifiez votre connexion et réessayez.</t>
         </is>
       </c>
       <c r="L62" s="4" t="inlineStr"/>
@@ -3869,7 +3861,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>codes.AI_PROVIDER_AUTH_FAILED</t>
+          <t>codes.TOO_MANY_SCANS</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -3879,30 +3871,30 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+          <t>You are sending scans too quickly. Wait a minute, then try again.</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+          <t>Kana aika bincike da sauri sosai. Jira minti ɗaya, sannan ka sake gwadawa.</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr"/>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+          <t>O ń fi àyẹ̀wò ránṣẹ́ ní kíákíá jù. Dúró fún ìṣẹ́jú kan, lẹ́yìn náà gbìyànjú lẹ́ẹ̀kan sí i.</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+          <t>Ị na-eziga nyocha ngwa ngwa. Chere otu nkeji, wee nwaa ọzọ.</t>
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr"/>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+          <t>Vous envoyez des analyses trop rapidement. Attendez une minute, puis réessayez.</t>
         </is>
       </c>
       <c r="L63" s="4" t="inlineStr"/>
@@ -3925,7 +3917,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>codes.AI_PROVIDER_NO_CREDIT</t>
+          <t>codes.INTERNAL_ERROR</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -3935,30 +3927,30 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+          <t>Something went wrong on our side. Your scan was NOT counted. Please try again, and contact support with the reference below if it keeps happening.</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+          <t>Wani abu ya lalace a ɓangarenmu. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa, kuma ka tuntuɓi tallafi da lambar shaida da ke ƙasa idan ya ci gaba.</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr"/>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+          <t>Nǹkan kan ṣẹlẹ̀ ní ẹ̀gbẹ́ wa. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i, kí o sì kàn sí ìrànlọ́wọ́ pẹ̀lú ìtọ́kasí ní ìsàlẹ̀ tí ó bá ń ṣẹlẹ̀ síbẹ̀.</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+          <t>Ihe ọjọọ mere n'akụkụ anyị. A GỤGHỊ nyocha gị. Biko nwaa ọzọ, kpọtụrụ ndị nkwado jiri ntụaka dị n'okpuru ma ọ bụrụ na ọ na-eme ọzọ.</t>
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr"/>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+          <t>Un problème est survenu de notre côté. Votre analyse n'a PAS été comptée. Veuillez réessayer et contactez l'assistance avec la référence ci-dessous si le problème persiste.</t>
         </is>
       </c>
       <c r="L64" s="4" t="inlineStr"/>
@@ -3981,7 +3973,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>codes.AI_PROVIDER_RATE_LIMIT</t>
+          <t>codes.ENGINE_UNREACHABLE</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -4037,7 +4029,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>codes.AI_PROVIDER_ERROR</t>
+          <t>codes.ENGINE_AUTH_FAILED</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -4085,8 +4077,232 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>app-errors</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>codes.AI_PROVIDER_AUTH_FAILED</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+        </is>
+      </c>
+      <c r="L67" s="4" t="inlineStr"/>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>(not in the app)</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>app-errors</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>codes.AI_PROVIDER_NO_CREDIT</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr"/>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr"/>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="inlineStr"/>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>(not in the app)</t>
+        </is>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>app-errors</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>codes.AI_PROVIDER_RATE_LIMIT</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr"/>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>(not in the app)</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>app-errors</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>codes.AI_PROVIDER_ERROR</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Our analysis service is temporarily unavailable. Your scan was NOT counted. Please try again in a few minutes.</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Sabis ɗin bincikenmu ba ya aiki na ɗan lokaci. BA a ƙirga binciken ka ba. Don Allah ka sake gwadawa nan da 'yan mintuna.</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr"/>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Iṣẹ́ àyẹ̀wò wa kò sí fún ìgbà díẹ̀. A KÒ ka àyẹ̀wò rẹ. Jọ̀wọ́ gbìyànjú lẹ́ẹ̀kan sí i lẹ́yìn ìṣẹ́jú díẹ̀.</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr"/>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>Ọrụ nyocha anyị adịghị ugbu a. A GỤGHỊ nyocha gị. Biko nwaa ọzọ n'ime nkeji ole na ole.</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr"/>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>Notre service d'analyse est temporairement indisponible. Votre analyse n'a PAS été comptée. Veuillez réessayer dans quelques minutes.</t>
+        </is>
+      </c>
+      <c r="L70" s="4" t="inlineStr"/>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>(not in the app)</t>
+        </is>
+      </c>
+      <c r="N70" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N66"/>
+  <autoFilter ref="A1:N70"/>
   <dataValidations count="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>